<commit_message>
Ajout de la route adminRoutes dans app.ts
</commit_message>
<xml_diff>
--- a/Template_Questions.xlsx
+++ b/Template_Questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F39D8B3-3B45-4FA4-86B1-8CA7495104E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9E2342-9071-45EC-9817-A2F223F42E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="144">
   <si>
     <t>Option 1</t>
   </si>
@@ -99,9 +99,6 @@
     <t>Biologie</t>
   </si>
   <si>
-    <t>ENSAM 2025</t>
-  </si>
-  <si>
     <t>Pascal</t>
   </si>
   <si>
@@ -172,15 +169,6 @@
   </si>
   <si>
     <t>Travail</t>
-  </si>
-  <si>
-    <t>FST 2025</t>
-  </si>
-  <si>
-    <t>ENSA 2025</t>
-  </si>
-  <si>
-    <t>ISTA 2025</t>
   </si>
   <si>
     <t>PHYSIQUE</t>
@@ -6184,6 +6172,15 @@
   </si>
   <si>
     <t>(R//R, C//C)</t>
+  </si>
+  <si>
+    <t>MEDECINE 2023</t>
+  </si>
+  <si>
+    <t>MEDECINE 2024</t>
+  </si>
+  <si>
+    <t>MEDECINE 2025</t>
   </si>
 </sst>
 </file>
@@ -7135,7 +7132,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>13</v>
@@ -7150,9 +7147,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -7167,24 +7164,24 @@
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" t="s">
         <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" t="s">
-        <v>24</v>
+        <v>48</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>58</v>
       </c>
       <c r="J2" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
@@ -7199,24 +7196,24 @@
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="G3" t="s">
         <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" t="s">
         <v>49</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>58</v>
       </c>
       <c r="J3" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -7231,24 +7228,24 @@
         <v>7</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G4" t="s">
         <v>5</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
-      </c>
-      <c r="I4" t="s">
         <v>50</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>58</v>
       </c>
       <c r="J4" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -7263,56 +7260,56 @@
         <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G5" t="s">
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
-      </c>
-      <c r="I5" t="s">
         <v>51</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>141</v>
       </c>
       <c r="J5" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
         <v>45</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>46</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>47</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" t="s">
         <v>48</v>
       </c>
-      <c r="F6" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" t="s">
-        <v>52</v>
-      </c>
-      <c r="I6" t="s">
-        <v>24</v>
+      <c r="I6" s="7" t="s">
+        <v>141</v>
       </c>
       <c r="J6" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B7" s="4">
         <v>11</v>
@@ -7333,74 +7330,74 @@
         <v>11</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" t="s">
         <v>49</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>141</v>
       </c>
       <c r="J7" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
         <v>41</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>42</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>43</v>
       </c>
-      <c r="E8" t="s">
-        <v>44</v>
-      </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" t="s">
         <v>50</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>141</v>
       </c>
       <c r="J8" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
         <v>33</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>34</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>35</v>
       </c>
-      <c r="E9" t="s">
-        <v>36</v>
-      </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" t="s">
         <v>51</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>142</v>
       </c>
       <c r="J9" s="3">
         <v>3</v>
@@ -7408,63 +7405,63 @@
     </row>
     <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
         <v>25</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>26</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>27</v>
       </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="J10" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
         <v>29</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>30</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>31</v>
       </c>
-      <c r="E11" t="s">
-        <v>32</v>
-      </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H11" t="s">
-        <v>54</v>
-      </c>
-      <c r="I11" t="s">
-        <v>24</v>
+        <v>50</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>142</v>
       </c>
       <c r="J11" s="3">
         <v>1</v>
@@ -7472,7 +7469,7 @@
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B12" s="4">
         <v>3</v>
@@ -7493,10 +7490,10 @@
         <v>15</v>
       </c>
       <c r="H12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="J12" s="3">
         <v>3</v>
@@ -7504,31 +7501,31 @@
     </row>
     <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
         <v>37</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>38</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>39</v>
       </c>
-      <c r="E13" t="s">
-        <v>40</v>
-      </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J13" s="3">
         <v>3</v>
@@ -7536,31 +7533,31 @@
     </row>
     <row r="14" spans="1:10" ht="63" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>61</v>
-      </c>
       <c r="G14" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J14" s="3">
         <v>2</v>
@@ -7568,31 +7565,31 @@
     </row>
     <row r="15" spans="1:10" ht="63" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="G15" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J15" s="3">
         <v>1</v>
@@ -7600,31 +7597,31 @@
     </row>
     <row r="16" spans="1:10" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="G16" s="5" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J16" s="3">
         <v>2</v>
@@ -7632,31 +7629,31 @@
     </row>
     <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>90</v>
-      </c>
       <c r="G17" s="11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J17" s="3">
         <v>3</v>
@@ -7664,31 +7661,31 @@
     </row>
     <row r="18" spans="1:10" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="F18" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>96</v>
-      </c>
       <c r="G18" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J18" s="3">
         <v>2</v>
@@ -7696,31 +7693,31 @@
     </row>
     <row r="19" spans="1:10" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="F19" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>102</v>
-      </c>
       <c r="G19" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J19" s="3">
         <v>1</v>
@@ -7728,31 +7725,31 @@
     </row>
     <row r="20" spans="1:10" ht="126" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="F20" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>108</v>
-      </c>
       <c r="G20" s="15" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J20" s="3">
         <v>1</v>
@@ -7760,31 +7757,31 @@
     </row>
     <row r="21" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="F21" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="C21" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>114</v>
-      </c>
       <c r="G21" s="13" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J21" s="3">
         <v>3</v>
@@ -7792,31 +7789,31 @@
     </row>
     <row r="22" spans="1:10" ht="63" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J22" s="3">
         <v>2</v>
@@ -7824,31 +7821,31 @@
     </row>
     <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="F23" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>123</v>
-      </c>
       <c r="G23" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>62</v>
+        <v>143</v>
       </c>
       <c r="J23" s="3">
         <v>2</v>
@@ -7856,31 +7853,31 @@
     </row>
     <row r="24" spans="1:10" ht="330.75" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D24" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>143</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="G24" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>62</v>
       </c>
       <c r="J24" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Fix Excel import propagation (exam/subject)
</commit_message>
<xml_diff>
--- a/Template_Questions.xlsx
+++ b/Template_Questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E521385-F8B0-490E-9396-28425CC6B1BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9126BCEA-8BBB-45DA-8925-43214C8372E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="223">
   <si>
     <t>Option 1</t>
   </si>
@@ -11767,6 +11767,18 @@
   </si>
   <si>
     <t>Q21M21</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>SIMPLE</t>
+  </si>
+  <si>
+    <t>GROUP</t>
+  </si>
+  <si>
+    <t>QUESTION</t>
   </si>
 </sst>
 </file>
@@ -12452,7 +12464,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -12486,11 +12498,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -12620,6 +12658,44 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12924,1291 +13000,1396 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="57.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="9" width="14.85546875" customWidth="1"/>
-    <col min="10" max="10" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="57.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="11" max="11" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B1" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
+    <row r="2" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B2" s="46" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="39"/>
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="K2" s="5">
+      <c r="L2" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="I3" s="42" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
     </row>
-    <row r="4" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+    <row r="4" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B4" s="46" t="s">
         <v>113</v>
       </c>
-      <c r="B4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="3"/>
+      <c r="D4" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="58" t="s">
         <v>61</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3"/>
+      <c r="K4" s="44"/>
+      <c r="L4" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="46" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="39"/>
+      <c r="D7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L7" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="6">
+        <v>11</v>
+      </c>
+      <c r="E8" s="6">
+        <v>13</v>
+      </c>
+      <c r="F8" s="6">
+        <v>15</v>
+      </c>
+      <c r="G8" s="6">
+        <v>17</v>
+      </c>
+      <c r="H8" s="6">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6">
+        <v>11</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="K4" s="5">
+      <c r="K8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L8" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
-        <v>114</v>
-      </c>
-      <c r="B5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="3" t="s">
+    <row r="9" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="39"/>
+      <c r="D9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="L9" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L10" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L11" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12" s="39"/>
+      <c r="D12" s="6">
+        <v>3</v>
+      </c>
+      <c r="E12" s="6">
         <v>5</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="F12" s="6">
+        <v>15</v>
+      </c>
+      <c r="G12" s="6">
+        <v>8</v>
+      </c>
+      <c r="H12" s="6">
+        <v>23</v>
+      </c>
+      <c r="I12" s="6">
+        <v>15</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L12" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="63" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B13" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="40"/>
+      <c r="D13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="K5" s="5">
-        <v>3</v>
+      <c r="K13" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="L13" s="5">
+        <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="39" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="44" t="s">
-        <v>136</v>
-      </c>
-      <c r="K6" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
-        <v>116</v>
-      </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="K7" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="B8" s="39"/>
-      <c r="C8" s="6">
-        <v>11</v>
-      </c>
-      <c r="D8" s="6">
-        <v>13</v>
-      </c>
-      <c r="E8" s="6">
-        <v>15</v>
-      </c>
-      <c r="F8" s="6">
-        <v>17</v>
-      </c>
-      <c r="G8" s="6">
-        <v>25</v>
-      </c>
-      <c r="H8" s="6">
-        <v>11</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="K8" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="39" t="s">
-        <v>118</v>
-      </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="K9" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="K10" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="K11" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="39" t="s">
-        <v>121</v>
-      </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="6">
-        <v>3</v>
-      </c>
-      <c r="D12" s="6">
-        <v>5</v>
-      </c>
-      <c r="E12" s="6">
-        <v>15</v>
-      </c>
-      <c r="F12" s="6">
-        <v>8</v>
-      </c>
-      <c r="G12" s="6">
-        <v>23</v>
-      </c>
-      <c r="H12" s="6">
-        <v>15</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="K12" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="63" x14ac:dyDescent="0.25">
-      <c r="A13" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="K13" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="63" x14ac:dyDescent="0.25">
-      <c r="A14" s="41" t="s">
+    <row r="14" spans="1:12" ht="63" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="41"/>
+      <c r="D14" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="E14" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="F14" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="G14" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="K14" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K14" s="5">
+      <c r="L14" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="41" t="s">
+    <row r="15" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B15" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="B15" s="41"/>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="41"/>
+      <c r="D15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="E15" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="G15" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="H15" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="I15" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="J15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="K15" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K15" s="5">
+      <c r="L15" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B16" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="10" t="s">
-        <v>72</v>
-      </c>
+      <c r="C16" s="9"/>
       <c r="D16" s="10" t="s">
         <v>72</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="G16" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="I16" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="J16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="K16" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K16" s="5">
+      <c r="L16" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B17" s="49" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="9"/>
+      <c r="D17" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>81</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="J17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="K17" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K17" s="5">
+      <c r="L17" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7"/>
+      <c r="D18" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="E18" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="F18" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="H18" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="I18" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="J18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="K18" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K18" s="5">
+      <c r="L18" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="126" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:12" ht="126" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B19" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="7"/>
+      <c r="D19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="E19" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="F19" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="J19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K19" s="5">
+      <c r="L19" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B20" s="50" t="s">
         <v>94</v>
       </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7"/>
+      <c r="D20" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="E20" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="F20" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="G20" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="G20" s="8" t="s">
+      <c r="H20" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="I20" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="J20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="K20" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K20" s="5">
+      <c r="L20" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B21" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="7"/>
+      <c r="D21" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="E21" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="F21" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="G21" s="11" t="s">
         <v>124</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>102</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="J21" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="K21" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K21" s="5">
+      <c r="L21" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+    <row r="22" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B22" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="8"/>
+      <c r="D22" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="F22" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="G22" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="H22" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="I22" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="J22" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="K22" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K22" s="5">
+      <c r="L22" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="283.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="37" t="s">
+    <row r="23" spans="1:12" ht="283.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B23" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="37"/>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="37"/>
+      <c r="D23" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="E23" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="F23" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="G23" s="12" t="s">
         <v>127</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>111</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="J23" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="K23" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K23" s="5">
+      <c r="L23" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="13"/>
+      <c r="D24" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="E24" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="F24" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="G24" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="G24" s="14" t="s">
+      <c r="H24" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="H24" s="14" t="s">
+      <c r="I24" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="J24" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J24" s="15" t="s">
+      <c r="K24" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K24" s="16">
+      <c r="L24" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" s="53" t="s">
         <v>203</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="13"/>
+      <c r="D25" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="E25" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="F25" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="G25" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="G25" s="17" t="s">
+      <c r="H25" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="H25" s="14" t="s">
+      <c r="I25" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="I25" s="15" t="s">
+      <c r="J25" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J25" s="15" t="s">
+      <c r="K25" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K25" s="16">
+      <c r="L25" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B26" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="13"/>
+      <c r="D26" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="E26" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="F26" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="G26" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="H26" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="I26" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="J26" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J26" s="15" t="s">
+      <c r="K26" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K26" s="16">
+      <c r="L26" s="16">
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+    <row r="27" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B27" s="54" t="s">
         <v>205</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="14" t="s">
+      <c r="C27" s="19"/>
+      <c r="D27" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="E27" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="F27" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="G27" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="G27" s="14" t="s">
+      <c r="H27" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="H27" s="14" t="s">
+      <c r="I27" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="J27" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J27" s="15" t="s">
+      <c r="K27" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K27" s="16">
+      <c r="L27" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+    <row r="28" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B28" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="19"/>
+      <c r="D28" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="E28" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="G28" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="G28" s="21" t="s">
+      <c r="H28" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="H28" s="14" t="s">
+      <c r="I28" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="J28" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J28" s="15" t="s">
+      <c r="K28" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K28" s="16">
+      <c r="L28" s="16">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="105" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B29" s="53" t="s">
         <v>207</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="13"/>
+      <c r="D29" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="E29" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="F29" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="G29" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="G29" s="23" t="s">
+      <c r="H29" s="23" t="s">
         <v>160</v>
       </c>
-      <c r="H29" s="23" t="s">
+      <c r="I29" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="I29" s="15" t="s">
+      <c r="J29" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J29" s="15" t="s">
+      <c r="K29" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K29" s="16">
+      <c r="L29" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
+    <row r="30" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B30" s="54" t="s">
         <v>208</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="19"/>
+      <c r="D30" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="E30" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="E30" s="21" t="s">
+      <c r="F30" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="G30" s="23" t="s">
         <v>164</v>
-      </c>
-      <c r="G30" s="21" t="s">
-        <v>165</v>
       </c>
       <c r="H30" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="I30" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="J30" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J30" s="15" t="s">
+      <c r="K30" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K30" s="16">
+      <c r="L30" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B31" s="53" t="s">
         <v>209</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="13"/>
+      <c r="D31" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="E31" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="F31" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="G31" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="G31" s="21" t="s">
+      <c r="H31" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="H31" s="23" t="s">
+      <c r="I31" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="J31" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J31" s="15" t="s">
+      <c r="K31" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K31" s="16">
+      <c r="L31" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="90" x14ac:dyDescent="0.25">
-      <c r="A32" s="19" t="s">
+    <row r="32" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B32" s="54" t="s">
         <v>210</v>
       </c>
-      <c r="B32" s="19"/>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="19"/>
+      <c r="D32" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="E32" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="F32" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="G32" s="23" t="s">
         <v>174</v>
-      </c>
-      <c r="G32" s="21" t="s">
-        <v>175</v>
       </c>
       <c r="H32" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="J32" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J32" s="15" t="s">
+      <c r="K32" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K32" s="16">
+      <c r="L32" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="90" x14ac:dyDescent="0.25">
-      <c r="A33" s="25" t="s">
+    <row r="33" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B33" s="55" t="s">
         <v>211</v>
       </c>
-      <c r="B33" s="25"/>
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="25"/>
+      <c r="D33" s="26" t="s">
         <v>176</v>
       </c>
-      <c r="D33" s="26" t="s">
+      <c r="E33" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="F33" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F33" s="26" t="s">
+      <c r="G33" s="26" t="s">
         <v>179</v>
       </c>
-      <c r="G33" s="26" t="s">
+      <c r="H33" s="26" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="I33" s="26" t="s">
         <v>179</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="J33" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J33" s="15" t="s">
+      <c r="K33" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K33" s="16">
+      <c r="L33" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B34" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="19"/>
+      <c r="D34" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="E34" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="F34" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="G34" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="H34" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="H34" s="13" t="s">
+      <c r="I34" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="I34" s="15" t="s">
+      <c r="J34" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J34" s="15" t="s">
+      <c r="K34" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K34" s="16">
+      <c r="L34" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="70.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
+    <row r="35" spans="1:12" ht="70.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B35" s="54" t="s">
         <v>213</v>
       </c>
-      <c r="B35" s="19"/>
-      <c r="C35" s="27" t="s">
+      <c r="C35" s="19"/>
+      <c r="D35" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="D35" s="28" t="s">
+      <c r="E35" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="F35" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="F35" s="29" t="s">
+      <c r="G35" s="29" t="s">
         <v>189</v>
       </c>
-      <c r="G35" s="30" t="s">
+      <c r="H35" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="H35" s="28" t="s">
+      <c r="I35" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="J35" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J35" s="15" t="s">
+      <c r="K35" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K35" s="16">
+      <c r="L35" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="69.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+    <row r="36" spans="1:12" ht="69.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B36" s="54" t="s">
         <v>214</v>
       </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="26">
+      <c r="C36" s="19"/>
+      <c r="D36" s="26">
         <v>4</v>
       </c>
-      <c r="D36" s="26">
+      <c r="E36" s="26">
         <v>8</v>
       </c>
-      <c r="E36" s="31">
+      <c r="F36" s="31">
         <v>12</v>
       </c>
-      <c r="F36" s="32">
+      <c r="G36" s="32">
         <v>24</v>
       </c>
-      <c r="G36" s="26">
+      <c r="H36" s="26">
         <v>36</v>
       </c>
-      <c r="H36" s="26">
+      <c r="I36" s="26">
         <v>4</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="J36" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J36" s="15" t="s">
+      <c r="K36" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K36" s="16">
+      <c r="L36" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="105" x14ac:dyDescent="0.25">
-      <c r="A37" s="33" t="s">
+    <row r="37" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B37" s="56" t="s">
         <v>215</v>
       </c>
-      <c r="B37" s="33"/>
-      <c r="C37" s="34" t="s">
+      <c r="C37" s="33"/>
+      <c r="D37" s="34" t="s">
         <v>191</v>
       </c>
-      <c r="D37" s="35" t="s">
+      <c r="E37" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="E37" s="34" t="s">
+      <c r="F37" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="F37" s="35" t="s">
+      <c r="G37" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="G37" s="34" t="s">
+      <c r="H37" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="H37" s="34" t="s">
+      <c r="I37" s="34" t="s">
         <v>191</v>
       </c>
-      <c r="I37" s="15" t="s">
+      <c r="J37" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J37" s="15" t="s">
+      <c r="K37" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K37" s="16">
+      <c r="L37" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="105" x14ac:dyDescent="0.25">
-      <c r="A38" s="36" t="s">
+    <row r="38" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B38" s="57" t="s">
         <v>216</v>
       </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="26" t="s">
+      <c r="C38" s="36"/>
+      <c r="D38" s="26" t="s">
         <v>196</v>
       </c>
-      <c r="D38" s="26" t="s">
+      <c r="E38" s="26" t="s">
         <v>197</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="F38" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="F38" s="26" t="s">
+      <c r="G38" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="G38" s="26" t="s">
+      <c r="H38" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="H38" s="26" t="s">
+      <c r="I38" s="26" t="s">
         <v>196</v>
       </c>
-      <c r="I38" s="15" t="s">
+      <c r="J38" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J38" s="15" t="s">
+      <c r="K38" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K38" s="37">
+      <c r="L38" s="37">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A39" s="37" t="s">
+    <row r="39" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B39" s="52" t="s">
         <v>217</v>
       </c>
-      <c r="B39" s="37"/>
-      <c r="C39" s="38">
+      <c r="C39" s="37"/>
+      <c r="D39" s="38">
         <v>0.08</v>
       </c>
-      <c r="D39" s="38">
+      <c r="E39" s="38">
         <v>0.16</v>
       </c>
-      <c r="E39" s="38">
+      <c r="F39" s="38">
         <v>0.32</v>
       </c>
-      <c r="F39" s="38">
+      <c r="G39" s="38">
         <v>0.64</v>
       </c>
-      <c r="G39" s="38">
+      <c r="H39" s="38">
         <v>0.96</v>
       </c>
-      <c r="H39" s="38">
+      <c r="I39" s="38">
         <v>0.32</v>
       </c>
-      <c r="I39" s="15" t="s">
+      <c r="J39" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="J39" s="15" t="s">
+      <c r="K39" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="K39" s="16">
+      <c r="L39" s="16">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel import + QCM display
</commit_message>
<xml_diff>
--- a/Template_Questions.xlsx
+++ b/Template_Questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9126BCEA-8BBB-45DA-8925-43214C8372E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B4EB59-82F8-4BE8-8FFE-DEBD19CCD290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="219">
   <si>
     <t>Option 1</t>
   </si>
@@ -11767,18 +11767,6 @@
   </si>
   <si>
     <t>Q21M21</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>SIMPLE</t>
-  </si>
-  <si>
-    <t>GROUP</t>
-  </si>
-  <si>
-    <t>QUESTION</t>
   </si>
 </sst>
 </file>
@@ -12464,7 +12452,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -12498,37 +12486,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -12658,44 +12620,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13000,1396 +12924,1291 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="57.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="57.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="3" max="3" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.85546875" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="B1" s="45" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>201</v>
+      </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>218</v>
+      </c>
+      <c r="I3" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="K3" s="43"/>
+    </row>
+    <row r="4" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="K4" s="5">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I5" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="K6" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A7" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="39"/>
+      <c r="C7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K7" s="5">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="8" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="C8" s="6">
+        <v>11</v>
+      </c>
+      <c r="D8" s="6">
+        <v>13</v>
+      </c>
+      <c r="E8" s="6">
+        <v>15</v>
+      </c>
+      <c r="F8" s="6">
+        <v>17</v>
+      </c>
+      <c r="G8" s="6">
+        <v>25</v>
+      </c>
+      <c r="H8" s="6">
+        <v>11</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K8" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" s="39"/>
+      <c r="C9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K9" s="5">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="2" t="s">
+    </row>
+    <row r="10" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="39"/>
+      <c r="C10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K10" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A11" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" s="39"/>
+      <c r="C11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K11" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" s="39"/>
+      <c r="C12" s="6">
+        <v>3</v>
+      </c>
+      <c r="D12" s="6">
+        <v>5</v>
+      </c>
+      <c r="E12" s="6">
         <v>15</v>
       </c>
+      <c r="F12" s="6">
+        <v>8</v>
+      </c>
+      <c r="G12" s="6">
+        <v>23</v>
+      </c>
+      <c r="H12" s="6">
+        <v>15</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K12" s="5">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B2" s="46" t="s">
-        <v>112</v>
-      </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="5">
+    <row r="13" spans="1:11" ht="63" x14ac:dyDescent="0.25">
+      <c r="A13" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="40"/>
+      <c r="C13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K13" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="L3" s="43"/>
-    </row>
-    <row r="4" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="58" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="58" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="58" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="58" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="I4" s="58" t="s">
-        <v>18</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="44"/>
-      <c r="L4" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B5" s="46" t="s">
-        <v>114</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="44"/>
-      <c r="L5" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>115</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="44"/>
-      <c r="L6" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="L7" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>117</v>
-      </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="6">
-        <v>11</v>
-      </c>
-      <c r="E8" s="6">
-        <v>13</v>
-      </c>
-      <c r="F8" s="6">
-        <v>15</v>
-      </c>
-      <c r="G8" s="6">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6">
-        <v>25</v>
-      </c>
-      <c r="I8" s="6">
-        <v>11</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="L8" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>118</v>
-      </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="L9" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B10" s="46" t="s">
-        <v>119</v>
-      </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L10" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B11" s="46" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L11" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="6">
-        <v>3</v>
-      </c>
-      <c r="E12" s="6">
-        <v>5</v>
-      </c>
-      <c r="F12" s="6">
-        <v>15</v>
-      </c>
-      <c r="G12" s="6">
-        <v>8</v>
-      </c>
-      <c r="H12" s="6">
-        <v>23</v>
-      </c>
-      <c r="I12" s="6">
-        <v>15</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L12" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L13" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B14" s="48" t="s">
+    <row r="14" spans="1:11" ht="63" x14ac:dyDescent="0.25">
+      <c r="A14" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="C14" s="41"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="8" t="s">
+        <v>50</v>
+      </c>
       <c r="D14" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>54</v>
+      <c r="I14" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J14" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K14" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="41" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="41"/>
+      <c r="C15" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="J15" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L14" s="5">
-        <v>1</v>
+      <c r="K15" s="5">
+        <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L15" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B16" s="49" t="s">
+    <row r="16" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="10" t="s">
+        <v>72</v>
+      </c>
       <c r="D16" s="10" t="s">
         <v>72</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G16" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="H16" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="H16" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>74</v>
+      <c r="I16" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K16" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L16" s="5">
+      <c r="K16" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B17" s="49" t="s">
+    <row r="17" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="D17" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="7" t="s">
         <v>80</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="9" t="s">
-        <v>81</v>
+      <c r="I17" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J17" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K17" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="J18" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L17" s="5">
-        <v>2</v>
+      <c r="K18" s="5">
+        <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B18" s="50" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L18" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="126" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B19" s="50" t="s">
+    <row r="19" spans="1:11" ht="126" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="D19" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="E19" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="F19" s="9" t="s">
         <v>92</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>93</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="I19" s="10" t="s">
-        <v>93</v>
+      <c r="I19" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J19" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K19" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="J20" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L19" s="5">
-        <v>1</v>
+      <c r="K20" s="5">
+        <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B20" s="50" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L20" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B21" s="50" t="s">
+    <row r="21" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="11" t="s">
+        <v>123</v>
+      </c>
       <c r="D21" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="F21" s="11" t="s">
         <v>124</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>102</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="I21" s="8" t="s">
-        <v>102</v>
+      <c r="I21" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J21" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K21" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="J22" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L21" s="5">
+      <c r="K22" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B22" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L22" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="283.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B23" s="52" t="s">
+    <row r="23" spans="1:11" ht="283.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="10" t="s">
+      <c r="B23" s="37"/>
+      <c r="C23" s="10" t="s">
         <v>110</v>
       </c>
+      <c r="D23" s="12" t="s">
+        <v>125</v>
+      </c>
       <c r="E23" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="G23" s="12" t="s">
         <v>127</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="I23" s="10" t="s">
-        <v>111</v>
+      <c r="I23" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="J23" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="K23" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="I24" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K23" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L23" s="5">
+      <c r="J24" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K24" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B24" s="53" t="s">
-        <v>202</v>
-      </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="J24" s="15" t="s">
+    <row r="25" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I25" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K24" s="15" t="s">
+      <c r="J25" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L24" s="16">
+      <c r="K25" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="B26" s="13"/>
+      <c r="C26" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K26" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="I27" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K27" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20" t="s">
+        <v>152</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="G28" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="H28" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K28" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="13"/>
+      <c r="C29" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="G29" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="H29" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K29" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B25" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="H25" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K25" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L25" s="16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B26" s="53" t="s">
-        <v>204</v>
-      </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="G26" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="H26" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="I26" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L26" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B27" s="54" t="s">
-        <v>205</v>
-      </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="J27" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K27" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L27" s="16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B28" s="54" t="s">
-        <v>206</v>
-      </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="G28" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="H28" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L28" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B29" s="53" t="s">
-        <v>207</v>
-      </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="E29" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="F29" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="H29" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="I29" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="J29" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K29" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L29" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B30" s="54" t="s">
+    <row r="30" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="C30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="21" t="s">
+        <v>161</v>
+      </c>
       <c r="D30" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="F30" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="F30" s="23" t="s">
         <v>164</v>
+      </c>
+      <c r="G30" s="21" t="s">
+        <v>165</v>
       </c>
       <c r="H30" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="I30" s="21" t="s">
-        <v>165</v>
+      <c r="I30" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="J30" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K30" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B31" s="13"/>
+      <c r="C31" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="F31" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="H31" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="I31" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K30" s="15" t="s">
+      <c r="J31" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L30" s="16">
+      <c r="K31" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B31" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="F31" s="23" t="s">
-        <v>168</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="H31" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="I31" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="J31" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K31" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L31" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="90" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B32" s="54" t="s">
+    <row r="32" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A32" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="24" t="s">
+      <c r="B32" s="19"/>
+      <c r="C32" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="D32" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="F32" s="21" t="s">
+      <c r="E32" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="G32" s="23" t="s">
+      <c r="F32" s="23" t="s">
         <v>174</v>
+      </c>
+      <c r="G32" s="21" t="s">
+        <v>175</v>
       </c>
       <c r="H32" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="I32" s="21" t="s">
-        <v>175</v>
+      <c r="I32" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="J32" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K32" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A33" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="B33" s="25"/>
+      <c r="C33" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="D33" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>179</v>
+      </c>
+      <c r="G33" s="26" t="s">
+        <v>180</v>
+      </c>
+      <c r="H33" s="26" t="s">
+        <v>179</v>
+      </c>
+      <c r="I33" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K32" s="15" t="s">
+      <c r="J33" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L32" s="16">
+      <c r="K33" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="90" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B33" s="55" t="s">
-        <v>211</v>
-      </c>
-      <c r="C33" s="25"/>
-      <c r="D33" s="26" t="s">
-        <v>176</v>
-      </c>
-      <c r="E33" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="F33" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="I33" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="J33" s="15" t="s">
+    <row r="34" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="H34" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="I34" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K33" s="15" t="s">
+      <c r="J34" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L33" s="16">
+      <c r="K34" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="70.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B35" s="19"/>
+      <c r="C35" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="G35" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="H35" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K35" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="69.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B36" s="19"/>
+      <c r="C36" s="26">
+        <v>4</v>
+      </c>
+      <c r="D36" s="26">
+        <v>8</v>
+      </c>
+      <c r="E36" s="31">
+        <v>12</v>
+      </c>
+      <c r="F36" s="32">
+        <v>24</v>
+      </c>
+      <c r="G36" s="26">
+        <v>36</v>
+      </c>
+      <c r="H36" s="26">
+        <v>4</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K36" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B34" s="54" t="s">
-        <v>212</v>
-      </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="I34" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="J34" s="15" t="s">
+    <row r="37" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="A37" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="D37" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="E37" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="F37" s="35" t="s">
+        <v>194</v>
+      </c>
+      <c r="G37" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="H37" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="I37" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K34" s="15" t="s">
+      <c r="J37" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L34" s="16">
+      <c r="K37" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="70.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B35" s="54" t="s">
-        <v>213</v>
-      </c>
-      <c r="C35" s="19"/>
-      <c r="D35" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="E35" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="F35" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="G35" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="H35" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="J35" s="15" t="s">
+    <row r="38" spans="1:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="A38" s="36" t="s">
+        <v>216</v>
+      </c>
+      <c r="B38" s="36"/>
+      <c r="C38" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>200</v>
+      </c>
+      <c r="H38" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="I38" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K35" s="15" t="s">
+      <c r="J38" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L35" s="16">
+      <c r="K38" s="37">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="69.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B36" s="54" t="s">
-        <v>214</v>
-      </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="26">
-        <v>4</v>
-      </c>
-      <c r="E36" s="26">
-        <v>8</v>
-      </c>
-      <c r="F36" s="31">
-        <v>12</v>
-      </c>
-      <c r="G36" s="32">
-        <v>24</v>
-      </c>
-      <c r="H36" s="26">
-        <v>36</v>
-      </c>
-      <c r="I36" s="26">
-        <v>4</v>
-      </c>
-      <c r="J36" s="15" t="s">
+    <row r="39" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="B39" s="37"/>
+      <c r="C39" s="38">
+        <v>0.08</v>
+      </c>
+      <c r="D39" s="38">
+        <v>0.16</v>
+      </c>
+      <c r="E39" s="38">
+        <v>0.32</v>
+      </c>
+      <c r="F39" s="38">
+        <v>0.64</v>
+      </c>
+      <c r="G39" s="38">
+        <v>0.96</v>
+      </c>
+      <c r="H39" s="38">
+        <v>0.32</v>
+      </c>
+      <c r="I39" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="K36" s="15" t="s">
+      <c r="J39" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L36" s="16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B37" s="56" t="s">
-        <v>215</v>
-      </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="34" t="s">
-        <v>191</v>
-      </c>
-      <c r="E37" s="35" t="s">
-        <v>192</v>
-      </c>
-      <c r="F37" s="34" t="s">
-        <v>193</v>
-      </c>
-      <c r="G37" s="35" t="s">
-        <v>194</v>
-      </c>
-      <c r="H37" s="34" t="s">
-        <v>195</v>
-      </c>
-      <c r="I37" s="34" t="s">
-        <v>191</v>
-      </c>
-      <c r="J37" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K37" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L37" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B38" s="57" t="s">
-        <v>216</v>
-      </c>
-      <c r="C38" s="36"/>
-      <c r="D38" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="F38" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="G38" s="26" t="s">
-        <v>199</v>
-      </c>
-      <c r="H38" s="26" t="s">
-        <v>200</v>
-      </c>
-      <c r="I38" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="J38" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K38" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L38" s="37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B39" s="52" t="s">
-        <v>217</v>
-      </c>
-      <c r="C39" s="37"/>
-      <c r="D39" s="38">
-        <v>0.08</v>
-      </c>
-      <c r="E39" s="38">
-        <v>0.16</v>
-      </c>
-      <c r="F39" s="38">
-        <v>0.32</v>
-      </c>
-      <c r="G39" s="38">
-        <v>0.64</v>
-      </c>
-      <c r="H39" s="38">
-        <v>0.96</v>
-      </c>
-      <c r="I39" s="38">
-        <v>0.32</v>
-      </c>
-      <c r="J39" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K39" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L39" s="16">
+      <c r="K39" s="16">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: add pdf worker
</commit_message>
<xml_diff>
--- a/Template_Questions.xlsx
+++ b/Template_Questions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\VER_01_02_26\MED-CONTEST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C8CDE0-A403-4AB2-A6CC-7A2AF6D12FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C2C200-5F6C-4B7E-B2D9-96767F319AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="224">
   <si>
     <t>Option 1</t>
   </si>
@@ -11779,6 +11779,9 @@
   </si>
   <si>
     <t>QUESTION</t>
+  </si>
+  <si>
+    <t>IM22-11</t>
   </si>
 </sst>
 </file>
@@ -12528,7 +12531,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -12696,6 +12699,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13000,7 +13004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="57.28515625" bestFit="1" customWidth="1"/>
@@ -14399,6 +14403,44 @@
         <v>2</v>
       </c>
     </row>
+    <row r="40" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="59" t="s">
+        <v>220</v>
+      </c>
+      <c r="B40" t="s">
+        <v>223</v>
+      </c>
+      <c r="C40" t="s">
+        <v>223</v>
+      </c>
+      <c r="D40" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="G40" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="H40" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="I40" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="K40" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="L40" s="16">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
fix : add pdf worker
</commit_message>
<xml_diff>
--- a/Template_Questions.xlsx
+++ b/Template_Questions.xlsx
@@ -5,18 +5,29 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MOULAY\Desktop\WEB_TEST_APP\MED-CONTEST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamch\OneDrive\Desktop\TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345CF74E-2E03-48EE-BC44-644174188C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B378B1-BAB7-423B-AE2C-473F9FE1EF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="383">
   <si>
     <t>Option 1</t>
   </si>
@@ -121,30 +132,6 @@
   </si>
   <si>
     <t>Rate</t>
-  </si>
-  <si>
-    <t>Inflammation</t>
-  </si>
-  <si>
-    <t>hypertension</t>
-  </si>
-  <si>
-    <t>glycémie</t>
-  </si>
-  <si>
-    <t>infection</t>
-  </si>
-  <si>
-    <t>Puissance</t>
-  </si>
-  <si>
-    <t>Energie</t>
-  </si>
-  <si>
-    <t>Force</t>
-  </si>
-  <si>
-    <t>Travail</t>
   </si>
   <si>
     <t>PHYSIQUE</t>
@@ -1542,12 +1529,6 @@
   </si>
   <si>
     <t>Physiologie</t>
-  </si>
-  <si>
-    <t>Pression</t>
-  </si>
-  <si>
-    <t>Huminité</t>
   </si>
   <si>
     <t>Bernard</t>
@@ -5959,15 +5940,6 @@
   </si>
   <si>
     <t>Quelle est la différence entre la souris et le rat ?</t>
-  </si>
-  <si>
-    <t>Dimension de R.T</t>
-  </si>
-  <si>
-    <t>plus petit nombre premier supérieur à 10</t>
-  </si>
-  <si>
-    <t>PCR</t>
   </si>
   <si>
     <t>Auteur de la théorie de réaction dans l'eau</t>
@@ -11781,9 +11753,6 @@
     <t>QUESTION</t>
   </si>
   <si>
-    <t>$\lim\below{n\rightarrow\infty}{\frac{b-a}{n}\ \sum_{k=0}^{n-1}{f\left(a+k\frac{b-a}{n}\right)=\ \lim\below{n\rightarrow\infty}{\frac{b-a}{n}\ \sum_{k=1}^{n}{f\left(a+k\frac{b-a}{n}\right)=\ \int_{a}^{b}f\left(x\right)dx}}\ }}$</t>
-  </si>
-  <si>
     <t>$\lim\below{n\rightarrow\infty}{U_n=\ -\infty}$</t>
   </si>
   <si>
@@ -11803,6 +11772,530 @@
   </si>
   <si>
     <t>Q22M22</t>
+  </si>
+  <si>
+    <t>(A) : $𝒛=√𝟏𝟎+𝟓√𝟐𝟐−𝒊√𝟏𝟎−𝟓√𝟐𝟐$</t>
+  </si>
+  <si>
+    <t>(B) : $𝒛=√𝟐+√𝟐𝟐−𝒊√𝟐−√𝟐𝟐$</t>
+  </si>
+  <si>
+    <t>(C) : $𝒛=√𝟏𝟎+𝟓√𝟐𝟐+𝒊√𝟏𝟎−𝟓√𝟐𝟐$</t>
+  </si>
+  <si>
+    <t>(D) : $𝒛=√𝟐+√𝟐𝟐+𝒊√𝟐−√𝟐𝟐$</t>
+  </si>
+  <si>
+    <t>(E) : $𝒛=√𝟏𝟎+𝟓√𝟐𝟐−𝒊√𝟏𝟎+𝟓√𝟐𝟐$</t>
+  </si>
+  <si>
+    <t>$U_{\mathrm{n}}=\frac{1}{2}+\frac{1}{2^{2}}+\frac{1}{2^{3}}+\cdots+\frac{1}{2^{n}}$ et $\boldsymbol{\operatorname { l n }}\left(V_{\mathrm{n}}\right)=U_{\mathrm{n}} \boldsymbol{\operatorname { l n }}(2)$; alors :</t>
+  </si>
+  <si>
+    <t>Pour tout $n$ entier et $n \geq 1$, on pose: 
+$U_{\mathrm{n}}=\frac{1}{2}+\frac{1}{2^{2}}+\frac{1}{2^{3}}+\cdots+\frac{1}{2^{n}}$      et       $\boldsymbol{\operatorname { l n }}\left(V_{\mathrm{n}}\right)=U_{\mathrm{n}} \boldsymbol{\operatorname { l n }}(2)$;       alors :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(A): $\lim _{n \rightarrow+\infty} U_{n}=1$ et $\lim _{n \rightarrow+\infty} V_{n}=\ln (2)$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(B): $\lim _{n \rightarrow+\infty} U_{n}=\frac{1}{2}$ et $\lim _{n \rightarrow+\infty} V_{n}=\ln (2)$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(C): $\lim _{n \rightarrow+\infty} U_{n}=2$ et $\lim _{n \rightarrow+\infty} V_{n}=1$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(D): $\lim _{n \rightarrow+\infty} U_{n}=\frac{1}{2}$ et $\lim _{n \rightarrow+\infty} V_{n}=2$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(E): $\lim _{\mathbf{n} \rightarrow+\infty} \mathbf{U}_{\mathbf{n}}=\mathbf{1}$ et $\lim _{\mathbf{n} \rightarrow+\infty} V_{\mathbf{n}}=\mathbf{2}$</t>
+  </si>
+  <si>
+    <t>Soit $\mathbf{f}$ une fonction définie sur $] 0 ;+\infty\left[\operatorname{par}: \boldsymbol{f}(\boldsymbol{x})=\frac{\sqrt{\boldsymbol{x}}}{\sqrt{\boldsymbol{x}+\mathbf{2} \sqrt{\boldsymbol{x}}}}\right.$          Alors $\lim _{x \rightarrow 0^{+}} f(x)$ est égale à :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(B): $\mathbf{0}$;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(E): la limite n'existe pas</t>
+  </si>
+  <si>
+    <t>Soit $\mathbf{f}$ une fonction réelle tels que $\boldsymbol{f}(\mathbf{1})=\mathbf{3}$ et $\boldsymbol{f}^{\prime}(\mathbf{1})=-\mathbf{3}$      
+La courbe de la fonction f admet au point $\boldsymbol{A}(\mathbf{1} ; \mathbf{3})$ une tangente d'équation</t>
+  </si>
+  <si>
+    <t>Soit $\mathbf{g}$ une fonction définie sur $] 0 ;+\infty\left[\right.$ par $: \boldsymbol{g}(\boldsymbol{x})=\frac{(\mathbf{2 x})^{\boldsymbol{x}}}{\boldsymbol{x}^{\mathbf{2 x}}}$        Alors $\lim _{\mathbf{x} \rightarrow+\infty} \mathbf{g}(\mathbf{x})$ est égale à :</t>
+  </si>
+  <si>
+    <t>Soient $\mathbf{f}$ et $\mathbf{g}$ deux fonctions définies par : $\boldsymbol{f}(\boldsymbol{x})=\boldsymbol{\operatorname { l n }}(\boldsymbol{x}-\mathbf{1})$ et $\boldsymbol{g}(\boldsymbol{x})=\sqrt{\boldsymbol{x}+\mathbf{1}}$    Alors le domaine de définition de gof est</t>
+  </si>
+  <si>
+    <t>Dans $\mathbb{C}$, si $\mathrm{z}=\sqrt{5} e^{-i \frac{\pi}{8}}$ alors :</t>
+  </si>
+  <si>
+    <t>Le nombre complexe $z=\left(\frac{1}{\sqrt{2}}(1-i \sqrt{3})\right)^{18}$ est égale à :</t>
+  </si>
+  <si>
+    <t>Pour $z \in \mathbb{C}-\{1\}$, l'ensemble des points $M$ d'affixe $z$ tels que $\frac{z+1}{z-1} \in i \mathbb{R}$ est :</t>
+  </si>
+  <si>
+    <t>Pour tout $n$ entier et $n \geq 2$, on pose: $$U_{n}=\left(1-\frac{1}{2^{2}}\right) \times\left(1-\frac{1}{3^{2}}\right) \times \ldots \times\left(1-\frac{1}{n^{2}}\right)$$    Alors $\lim _{n \rightarrow+\infty} U_{n}$ est égale à :</t>
+  </si>
+  <si>
+    <t>(A) $: Z=\frac{\sqrt{10+5 \sqrt{2}}}{2}-\frac{i \sqrt{10-5 \sqrt{2}}}{2}$</t>
+  </si>
+  <si>
+    <t>(B) $: Z=\frac{\sqrt{2+\sqrt{2}}}{2}-\frac{i \sqrt{2-\sqrt{2}}}{2}$</t>
+  </si>
+  <si>
+    <t>(C) $: Z=\frac{\sqrt{10+5 \sqrt{2}}}{2}+\frac{i \sqrt{10-5 \sqrt{2}}}{2}$</t>
+  </si>
+  <si>
+    <t>(D) $: z=\frac{\sqrt{2+\sqrt{2}}}{2}+\frac{i \sqrt{2-\sqrt{2}}}{2}$</t>
+  </si>
+  <si>
+    <t>(E): $Z=\frac{\sqrt{10+5 \sqrt{2}}}{2}-\frac{i \sqrt{10+5 \sqrt{2}}}{2}$</t>
+  </si>
+  <si>
+    <t>(E): $z=\frac{1}{2}-i \frac{\sqrt{3}}{2}$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{C}):+\infty$</t>
+  </si>
+  <si>
+    <t>(E): la limite n'existe pas</t>
+  </si>
+  <si>
+    <t>L'intégrale $\int_{\frac{\pi}{6}}^{\frac{\pi}{4}} \frac{1}{\sin (x) \tan (x)}$ dx est égale à :</t>
+  </si>
+  <si>
+    <t>L'intégrale $\int_{0}^{\frac{\pi}{2}} \frac{\sin (2 \mathrm{x})}{1+\sin ^{2}(x)} \mathrm{dx}$ est égale à :</t>
+  </si>
+  <si>
+    <t>Soit f une fonction réelle définie par $f(x)=x+x^{2} \sin \left(\frac{1}{x}\right)$ si $x \neq 0$ et $f(0)=0$    Alors :</t>
+  </si>
+  <si>
+    <t>$(A): 0$</t>
+  </si>
+  <si>
+    <t>$(B): \ln (2)+1$</t>
+  </si>
+  <si>
+    <t>$(C): \boldsymbol{f}^{\prime}(\mathbf{0})=\mathbf{1} \quad ;  \boldsymbol{\operatorname { s i n }}\left(\frac{\mathbf{1}}{\boldsymbol{x}}\right)+\boldsymbol{\operatorname { c o s }}\left(\frac{\mathbf{1}}{\boldsymbol{x}}\right)$</t>
+  </si>
+  <si>
+    <t>(E): $\boldsymbol{f}$ est dérivable en 0 et $\boldsymbol{f}^{\prime}(0)=2$</t>
+  </si>
+  <si>
+    <t>$(E): \frac{\mathbf{8} \times \mathbf{3}^{\boldsymbol{n}}}{\mathbf{1 1}^{\boldsymbol{n} \boldsymbol{-} \mathbf{1}}}$</t>
+  </si>
+  <si>
+    <t>(B): $z=\frac{\sqrt{3}}{2}-\frac{1}{2} i$</t>
+  </si>
+  <si>
+    <t>(A): z=-512</t>
+  </si>
+  <si>
+    <t>(C): z=512</t>
+  </si>
+  <si>
+    <t>(D): z=251</t>
+  </si>
+  <si>
+    <t>(C): Le cercle de centre $O$ et de rayon 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (D): la droite (Ox)</t>
+  </si>
+  <si>
+    <t>$(A): 1 \quad$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{B}): \quad \mathbf{0} \quad $</t>
+  </si>
+  <si>
+    <t>(D): $\frac{\mathbf{1}}{\mathbf{2}} \quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(A): $+\infty$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(B): $\mathbf{0}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(C): $\mathbf{1} \quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(D): $\frac{\mathbf{1}}{\mathbf{2}} \quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(B): 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(C): 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(D): $\mathbf{0} \quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+$(A): \mathbf{y}=\mathbf{3 x}-\mathbf{2}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+$(B): \mathbf{y}=\mathbf{3 x}-\mathbf{6}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+$(C): \mathbf{y}=-\mathbf{3 x}+\mathbf{6}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+$(E): \mathbf{y}=-\mathbf{3 x}+\mathbf{2}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(A): $[-\mathbf{1} ;+\infty[$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(B): $] \mathbf{1} ;+\infty[\quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(C) : $\left[\mathbf{1}+\frac{\mathbf{1}}{\boldsymbol{e}} ;+\infty[\right.$</t>
+  </si>
+  <si>
+    <t>(D): $\frac{\sqrt{\mathbf{2}}}{\mathbf{2}}-\frac{\mathbf{1}}{\mathbf{2}} \quad$</t>
+  </si>
+  <si>
+    <t>(A): $\frac{1}{2}-\frac{\sqrt{2}}{2}$</t>
+  </si>
+  <si>
+    <t>(B): $2-\sqrt{2}$</t>
+  </si>
+  <si>
+    <t>(C): $\sqrt{2}-2$</t>
+  </si>
+  <si>
+    <t>(C): $\ln (2) \quad$</t>
+  </si>
+  <si>
+    <t>(D): $1 \quad$</t>
+  </si>
+  <si>
+    <t>(E):$-\ln (2)$</t>
+  </si>
+  <si>
+    <t>Dans l'espace rapporté à un repère orthonormé $\operatorname{direct}(O, \vec{\imath}, \vec{\jmath}, \vec{k})$    Soit les plans $(P): x-y-z+2=0$ et $\left(P^{\prime}\right): x+z-2=0$ et la droite $(\Delta)$ telle que $\left\{\begin{array}{l}x=1+t;     \\ y=2+2 t;     \\ z=1-t\end{array} ;(t \in \mathbb{R})\right.$, alors :</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{A}):(\Delta) \subset(\boldsymbol{P})$</t>
+  </si>
+  <si>
+    <t>(A): $\frac{\mathbf{8} \times \mathbf{3}^{\boldsymbol{n}}}{\mathbf{1 1}^{\boldsymbol{n}}} \quad$</t>
+  </si>
+  <si>
+    <t>(B): $\frac{\mathbf{8 n} \times \mathbf{3}^{\boldsymbol{n}}}{\mathbf{1 1}^{\boldsymbol{n}}}$</t>
+  </si>
+  <si>
+    <t>(C): $\frac{8 n \times 3^{n-1}}{11^{n}} \quad$</t>
+  </si>
+  <si>
+    <t>(D): $\frac{\mathbf{8}^{\boldsymbol{n}} \times \mathbf{3}^{\boldsymbol{n - 1}}}{\mathbf{1 1}^{\boldsymbol{n}}}$</t>
+  </si>
+  <si>
+    <t>Une urne contient 5 boules bleus, 4 boules blanches et 3 boules noires. Les boules sont indiscernables au toucher.  On tire au hasard et simultanément 3 boules de ce sac, on répète cette expérience n fois de suite ( $n \geq  5$ ) en remettant dans l'urne les boules tirées après chaque tirage, La probabilité d'obtenir 3 boules de couleurs deux à deux distinctes ( $n-1$ ) fois exactement est :</t>
+  </si>
+  <si>
+    <t>$(C): \boldsymbol{f}^{\prime}(\mathbf{0})=\mathbf{1} \quad$</t>
+  </si>
+  <si>
+    <t>$(A): f$ est dérivable en $0 \quad$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{B}):(\Delta) \perp(\boldsymbol{P})$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{C}):(\Delta) \cap(\boldsymbol{P})=\emptyset$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{D}):(\Delta) \cap\left(\boldsymbol{P}^{\prime}\right)=\emptyset $</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{E}):(\Delta) \perp\left(\boldsymbol{P}^{\prime}\right)$</t>
+  </si>
+  <si>
+    <t>$\quad(\boldsymbol{E}): $\mathbf{1}-\sqrt{\mathbf{2}}$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(D): $] \boldsymbol{e} ;+\infty[\quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+(E): $] \boldsymbol{-e} ;+\infty[\quad$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+$(D): \mathbf{y}=\mathbf{3 x}$</t>
+  </si>
+  <si>
+    <t>(B) : La droite $(O y)$ privée du point (0,1)</t>
+  </si>
+  <si>
+    <t>(A) : La droite $(O x)$ privée du point (1,0)</t>
+  </si>
+  <si>
+    <t>(E) : Le cercle de centre $O$ et de rayon 1 privée du point (1,0)</t>
+  </si>
+  <si>
+    <t>$ (B): \mathbf{f}^{\prime}(\mathbf{0})=\mathbf{0}$</t>
+  </si>
+  <si>
+    <t>$(\boldsymbol{D}):\text{ Pour tout } \boldsymbol{x} \neq \mathbf{0}, \quad \boldsymbol{f}(\boldsymbol{x}) = \mathbf{1} + \mathbf{2}\boldsymbol{x}\sin\left(\frac{\mathbf{1}}{\boldsymbol{x}}\right) + \cos\left(\frac{\mathbf{1}}{\boldsymbol{x}}\right)$</t>
+  </si>
+  <si>
+    <t>Soit $I=\int_{0}^{\pi}|\cos x| d x$. Quelle est la valeur de $I$ ?</t>
+  </si>
+  <si>
+    <t>Quelle est la valeur de l'intégrale définie suivante : $J=\int_{0}^{1} \frac{1-x^{2}}{\left(1+x^{2}\right)^{2}}$</t>
+  </si>
+  <si>
+    <t>Soit la suite ( $U_{n}$ ) définie par : $U_{1}=1$ et pour tout $n \geq 1$,$$U_{n+1}=\sqrt{2+U_{n}}$$. Quelle est la limite de la suite ( $\boldsymbol{U}_{\boldsymbol{n}}$ ) ?</t>
+  </si>
+  <si>
+    <t>Soient $a$ et $b$ deux nombres complexes tels que : $a \neq b$ et $|a|=1$. Quelle est la valeur de :$$\left|\frac{a-b}{1-\bar{a} b}\right|$$</t>
+  </si>
+  <si>
+    <t>Soit $C=1+\cos \frac{\pi}{5}+\cos \frac{2 \pi}{5}+\cdots+\cos \frac{9 \pi}{5}$ et $S=\sin \frac{\pi}{5}+\sin \frac{2 \pi}{5}+\cdots+\sin \frac{9 \pi}{5}$. Quelle est la valeur de $\mathbf{z}=\mathbf{C}+\mathbf{i S}$.</t>
+  </si>
+  <si>
+    <t>Soit la fonction $\boldsymbol{f}(\boldsymbol{x})=\sin \boldsymbol{x}+\cos \boldsymbol{x}$. Quelle est la valeur maximale de $\mathbf{f}(\mathbf{x})$ sur $\mathbb{R}$ ?</t>
+  </si>
+  <si>
+    <t>Résoudre dans $R$ 1'équation : $\frac{e^{2 x-1}}{\sqrt{e^{2 x+4}}}=e^{-x}$. Quelle est la bonne réponse?</t>
+  </si>
+  <si>
+    <t>Une urne $U$ contient 9 boules : dont 5 boules rouges numérotées de 1 à 5 et 4 boule noires numérotées de 1 à 4 . On suppose que les boules sont indiscernables au toucher. On tire simultanément deux boules de l'urne. On considère les deux événements $A$ : « les deux boules tirées sont de mème couleur» et $B$ « les deux boules tirés portent un numéro pair». Calculer $\boldsymbol{P}_{\bar{A}}(\boldsymbol{B})$ ?</t>
+  </si>
+  <si>
+    <t>On lance deux dés équilibrés à 6 faces. Quelle est la probabilité d'obtenir au moins un 6 ?</t>
+  </si>
+  <si>
+    <t>Soient les points : $A(1,1,-2), B(0,5,5), C(6,-3,-5), D(1,2,0)$, Levecteur $\overrightarrow{A D}$ appartient-il au plan vectoriel engendré par $\overrightarrow{\mathrm{AB}} \boldsymbol{e} \boldsymbol{t}. Autrement dit, existe-t-il des réels $x$ et y tels que : $\overrightarrow{A D}=x \overrightarrow{A B}+y \overrightarrow{A C}$ ? \overrightarrow{\mathrm{AC}}$</t>
+  </si>
+  <si>
+    <t>Soient $\vec{u}(1,2,-1), \vec{v}(3,6,-3), \vec{w}(0,1,1)$. Quelle est la valeur de ce produit $(\overrightarrow{\boldsymbol{u}} \wedge \overrightarrow{\boldsymbol{v}}), \overrightarrow{\boldsymbol{w}}$</t>
+  </si>
+  <si>
+    <t>La fonction $f: f(x)=\frac{\ln (x+1)}{x+e^{x}}$ admet au point $0(0,0)$ une tangente d'équation :</t>
+  </si>
+  <si>
+    <t>On considère le nombre complexe : $z=(1+i)^{20}$ Quelle est la partie imaginaire de $z$ ?</t>
+  </si>
+  <si>
+    <t>(A): 0</t>
+  </si>
+  <si>
+    <t>(B): .1</t>
+  </si>
+  <si>
+    <t>(C): 2</t>
+  </si>
+  <si>
+    <t>(D): $\pi$</t>
+  </si>
+  <si>
+    <t>(E) : Aucune des réponses n'est juste</t>
+  </si>
+  <si>
+    <t>A) $\frac{1}{2}$</t>
+  </si>
+  <si>
+    <t>В) $\frac{\pi}{4}$</t>
+  </si>
+  <si>
+    <t>C) $\frac{1}{4}$</t>
+  </si>
+  <si>
+    <t>D) 0</t>
+  </si>
+  <si>
+    <t>E). Aucune des réponses n'est juste</t>
+  </si>
+  <si>
+    <t>A) $\sqrt{2}$</t>
+  </si>
+  <si>
+    <t>B) $\mathbf{1}+\sqrt{\mathbf{2}}$</t>
+  </si>
+  <si>
+    <t>C) la suite est divergente</t>
+  </si>
+  <si>
+    <t>D) 2</t>
+  </si>
+  <si>
+    <t>E) Aucune des réponses n'est juste</t>
+  </si>
+  <si>
+    <t>A) 0</t>
+  </si>
+  <si>
+    <t>B) 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> C) 2</t>
+  </si>
+  <si>
+    <t>D) $\sqrt{2}$</t>
+  </si>
+  <si>
+    <t>A) 1</t>
+  </si>
+  <si>
+    <t>B) 2</t>
+  </si>
+  <si>
+    <t>C) -1</t>
+  </si>
+  <si>
+    <t>А) 0</t>
+  </si>
+  <si>
+    <t>B) $\frac{1}{2}$</t>
+  </si>
+  <si>
+    <t>C) 1</t>
+  </si>
+  <si>
+    <t>D) -1</t>
+  </si>
+  <si>
+    <t>В) $\sqrt{2}+1$</t>
+  </si>
+  <si>
+    <t>C) 2</t>
+  </si>
+  <si>
+    <t>А) $x=1$</t>
+  </si>
+  <si>
+    <t>В) $x=0$</t>
+  </si>
+  <si>
+    <t>C) $x=\frac{3}{2}$</t>
+  </si>
+  <si>
+    <t>D) $x=-1$</t>
+  </si>
+  <si>
+    <t>A) $\frac{\mathbf{1}}{\mathbf{1 8}}$</t>
+  </si>
+  <si>
+    <t>B) $\frac{17}{18}$</t>
+  </si>
+  <si>
+    <t>C) $\frac{2}{9}$</t>
+  </si>
+  <si>
+    <t>D) $\frac{1}{5}$</t>
+  </si>
+  <si>
+    <t>E) Aucune des réponses $n^{\prime}$ est juste</t>
+  </si>
+  <si>
+    <t>A) $\frac{1}{6}$</t>
+  </si>
+  <si>
+    <t>В) $\frac{11}{36}$</t>
+  </si>
+  <si>
+    <t>C) $\frac{5}{36}$</t>
+  </si>
+  <si>
+    <t>D) $\frac{25}{36}$</t>
+  </si>
+  <si>
+    <t>A) Oui, pour $x=, \frac{1}{4}, y=, \frac{1}{8}$</t>
+  </si>
+  <si>
+    <t>B) oui, pour $x=\frac{5}{16}, y=\frac{1}{16}$</t>
+  </si>
+  <si>
+    <t>C) Oui, pour $x=\frac{1}{2}, y=\frac{1}{2}$</t>
+  </si>
+  <si>
+    <t>D) Non, car le vecteur $\overrightarrow{A D}$ n'est pas une combinaison linéaire de $\overrightarrow{A B}$ et $\overrightarrow{A C}$</t>
+  </si>
+  <si>
+    <t>B) 3</t>
+  </si>
+  <si>
+    <t>D. 2</t>
+  </si>
+  <si>
+    <t>А) $y=x$</t>
+  </si>
+  <si>
+    <t>В) $y=x+1$</t>
+  </si>
+  <si>
+    <t>C) $y=-2 x$</t>
+  </si>
+  <si>
+    <t>D) $y=x-1$</t>
+  </si>
+  <si>
+    <t>A) $2^{10}$</t>
+  </si>
+  <si>
+    <t>B) $-2^{10}$</t>
+  </si>
+  <si>
+    <t>C) 0</t>
+  </si>
+  <si>
+    <t>On définit la fonction : $f(x)=\left\{\begin{array}{l}\frac{\sqrt{1+x}-1}{x}, x \neq 0 \\      a, x=0\end{array}\right.$. Pour quelle valeur de $\boldsymbol{a}$ la fonction $\boldsymbol{f}$ est-elle continue en $\boldsymbol{x}=\mathbf{0}$ ?</t>
+  </si>
+  <si>
+    <t>\section*{Propagation d'une onde le long d'une corde : }.     Une lame vibrante horizontale, fixée à l'extrémité $S$ d'une corde élastique, génère le long de celle-ci une onde progressive sinusoïdale de célérité $\nu$. Le mouvement de $S$ débute à l'instant $t_{0}=0$. Les figures (1) et (2) ci-dessous représentent l'élongation d'un point $M$ de la corde, situé à une distance $d$ de $S$, et l'aspect de la corde à l'instant $t_{1}=0,16 \mathrm{~s}$. Le front d' onde se trouve à l'instant $t_{1}$ à la distance $S F=80 c m$ de $S$.</t>
+  </si>
+  <si>
+    <t>\begin{figure}      \includegraphics[alt={},max width=\textwidth]{https://cdn.mathpix.com/cropped/279e22aa-95a9-45ef-a751-9e3ff09a38fe-1.jpg?height=265&amp;width=939&amp;top_left_y=752&amp;top_left_x=133}     \captionsetup{labelformat=empty}       \caption{Figure 1}     \end{figure}    \begin{figure}     \includegraphics[alt={},max width=\textwidth]{https://cdn.mathpix.com/cropped/279e22aa-95a9-45ef-a751-9e3ff09a38fe-1.jpg?height=216&amp;width=552&amp;top_left_y=803&amp;top_left_x=1237}     \captionsetup{labelformat=empty}    \caption{Figure 2}      \end{figure}</t>
+  </si>
+  <si>
+    <t>Q21. Les valeurs de la longueur d'onde et de la célérité de propagation de l'onde le long de la corde sont :</t>
+  </si>
+  <si>
+    <t>$\mathbf{A}$ &amp; $\lambda=0,40 \mathrm{~m}$  \\ $v=0,25 \mathrm{~m} \cdot \mathrm{~s}^{-1}$</t>
+  </si>
+  <si>
+    <t>$\mathbf{B}$ &amp; $\lambda=0,08 \mathrm{~m}$  \\ $v=0,80 \mathrm{~m} \cdot \mathrm{~s}^{-1}$</t>
+  </si>
+  <si>
+    <t>$\mathbf{C}$ &amp; $\lambda=0,40 \mathrm{~m}$  \\ $\mathbf{C}$ &amp; $v=2,5 \mathrm{~m} \cdot \mathrm{~s}^{-1}$</t>
+  </si>
+  <si>
+    <t>$\mathbf{D}=0,40 \mathrm{~m}$  \\  $\mathbf{D}$ &amp; $v=5,0 \mathrm{~m} \cdot \mathrm{~s}^{-1}$</t>
+  </si>
+  <si>
+    <t>$\lambda=0,80 \mathrm{~m}$  \\ $\mathbf{E}$ &amp; $v=10 \mathrm{~m} \cdot \mathrm{~s}^{-1}$</t>
   </si>
 </sst>
 </file>
@@ -12488,7 +12981,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -12515,44 +13008,16 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -12673,54 +13138,31 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="70" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="97" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13025,7 +13467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="57.28515625" bestFit="1" customWidth="1"/>
@@ -13033,7 +13475,8 @@
     <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.140625" customWidth="1"/>
+    <col min="8" max="8" width="39.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="28.7109375" customWidth="1"/>
     <col min="10" max="10" width="14.85546875" customWidth="1"/>
     <col min="11" max="11" width="21.140625" customWidth="1"/>
@@ -13041,13 +13484,13 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="B1" s="45" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -13062,7 +13505,7 @@
         <v>3</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>13</v>
@@ -13079,10 +13522,10 @@
     </row>
     <row r="2" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B2" s="46" t="s">
-        <v>112</v>
+        <v>207</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>102</v>
       </c>
       <c r="C2" s="39"/>
       <c r="D2" s="3" t="s">
@@ -13098,16 +13541,16 @@
         <v>11</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="L2" s="5">
         <v>2</v>
@@ -13115,10 +13558,11 @@
     </row>
     <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>221</v>
-      </c>
+        <v>208</v>
+      </c>
+      <c r="B3" s="3"/>
       <c r="C3" s="3" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -13126,57 +13570,57 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="42" t="s">
-        <v>40</v>
+      <c r="J3" s="43" t="s">
+        <v>32</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="L3" s="43"/>
+        <v>123</v>
+      </c>
+      <c r="L3" s="44"/>
     </row>
     <row r="4" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>113</v>
+        <v>209</v>
+      </c>
+      <c r="B4" s="39" t="s">
+        <v>103</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D4" s="58" t="s">
+        <v>205</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="58" t="s">
+      <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="58" t="s">
+      <c r="F4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="58" t="s">
+      <c r="G4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="I4" s="58" t="s">
+      <c r="H4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="J4" s="3"/>
-      <c r="K4" s="44"/>
+      <c r="K4" s="42"/>
       <c r="L4" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B5" s="46" t="s">
-        <v>114</v>
+        <v>209</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>104</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>4</v>
@@ -13191,26 +13635,26 @@
         <v>7</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="J5" s="3"/>
-      <c r="K5" s="44"/>
+      <c r="K5" s="42"/>
       <c r="L5" s="5">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>115</v>
+        <v>209</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>105</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>20</v>
@@ -13225,48 +13669,48 @@
         <v>23</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>21</v>
       </c>
       <c r="J6" s="3"/>
-      <c r="K6" s="44"/>
+      <c r="K6" s="42"/>
       <c r="L6" s="5">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>116</v>
+        <v>207</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>106</v>
       </c>
       <c r="C7" s="39"/>
       <c r="D7" s="3" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="L7" s="5">
         <v>2</v>
@@ -13274,35 +13718,35 @@
     </row>
     <row r="8" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>117</v>
+        <v>207</v>
+      </c>
+      <c r="B8" s="39" t="s">
+        <v>107</v>
       </c>
       <c r="C8" s="39"/>
-      <c r="D8" s="6">
-        <v>11</v>
-      </c>
-      <c r="E8" s="6">
-        <v>13</v>
-      </c>
-      <c r="F8" s="6">
-        <v>15</v>
-      </c>
-      <c r="G8" s="6">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6">
-        <v>25</v>
-      </c>
-      <c r="I8" s="6">
-        <v>11</v>
+      <c r="D8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="L8" s="5">
         <v>1</v>
@@ -13310,1192 +13754,2175 @@
     </row>
     <row r="9" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>118</v>
+        <v>207</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>108</v>
       </c>
       <c r="C9" s="39"/>
-      <c r="D9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="D9" s="6">
+        <v>3</v>
+      </c>
+      <c r="E9" s="6">
+        <v>5</v>
+      </c>
+      <c r="F9" s="6">
+        <v>15</v>
+      </c>
+      <c r="G9" s="6">
+        <v>8</v>
+      </c>
+      <c r="H9" s="6">
+        <v>23</v>
+      </c>
+      <c r="I9" s="6">
+        <v>15</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>42</v>
-      </c>
       <c r="K9" s="4" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="L9" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="63" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B10" s="46" t="s">
-        <v>119</v>
-      </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>42</v>
+        <v>207</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="40"/>
+      <c r="D10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>34</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="L10" s="5">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="63" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B11" s="46" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J11" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="41"/>
+      <c r="D11" s="8" t="s">
         <v>42</v>
       </c>
+      <c r="E11" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="K11" s="4" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="L11" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B12" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="41"/>
+      <c r="D12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L12" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L13" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L14" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L15" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="126" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L16" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L17" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L18" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L19" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="283.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="37"/>
+      <c r="D20" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L20" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G21" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="6">
-        <v>3</v>
-      </c>
-      <c r="E12" s="6">
+      <c r="H21" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K21" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L21" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K22" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L22" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K23" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L23" s="16">
         <v>5</v>
-      </c>
-      <c r="F12" s="6">
-        <v>15</v>
-      </c>
-      <c r="G12" s="6">
-        <v>8</v>
-      </c>
-      <c r="H12" s="6">
-        <v>23</v>
-      </c>
-      <c r="I12" s="6">
-        <v>15</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="L12" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B13" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="40"/>
-      <c r="D13" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L13" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="63" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L14" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="41"/>
-      <c r="D15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L15" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B16" s="49" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L16" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B17" s="49" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L17" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B18" s="50" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L18" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="126" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B19" s="50" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K19" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L19" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B20" s="50" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="I20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L20" s="5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B21" s="50" t="s">
-        <v>100</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L21" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B22" s="51" t="s">
-        <v>103</v>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L22" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="283.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B23" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="L23" s="5">
-        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B24" s="53" t="s">
-        <v>202</v>
-      </c>
-      <c r="C24" s="13"/>
+        <v>207</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="C24" s="19"/>
       <c r="D24" s="14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J24" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K24" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L24" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="F25" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="L24" s="16">
+      <c r="G25" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="H25" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K25" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L25" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K26" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L26" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B25" s="53" t="s">
-        <v>203</v>
-      </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="H25" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K25" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L25" s="16">
+    <row r="27" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="C27" s="19"/>
+      <c r="D27" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="F27" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="H27" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="I27" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L27" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="H28" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="I28" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L28" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="G29" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="I29" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K29" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L29" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B26" s="53" t="s">
-        <v>204</v>
-      </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="G26" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="H26" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="I26" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K26" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L26" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B27" s="54" t="s">
-        <v>205</v>
-      </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="J27" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K27" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L27" s="16">
+    <row r="30" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="C30" s="25"/>
+      <c r="D30" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="G30" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="H30" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K30" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="L30" s="16">
         <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B28" s="54" t="s">
-        <v>206</v>
-      </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="G28" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="H28" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L28" s="16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B29" s="53" t="s">
-        <v>207</v>
-      </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="E29" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="F29" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="H29" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="I29" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="J29" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K29" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L29" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B30" s="54" t="s">
-        <v>208</v>
-      </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="F30" s="21" t="s">
-        <v>163</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="H30" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="I30" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="J30" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K30" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L30" s="16">
-        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B31" s="53" t="s">
-        <v>209</v>
-      </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="F31" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="23" t="s">
+      <c r="E31" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="H31" s="21" t="s">
+      <c r="F31" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="I31" s="23" t="s">
-        <v>166</v>
+      <c r="G31" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="H31" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>169</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K31" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L31" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" ht="70.5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B32" s="54" t="s">
-        <v>210</v>
+        <v>207</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>200</v>
       </c>
       <c r="C32" s="19"/>
-      <c r="D32" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="F32" s="21" t="s">
+      <c r="D32" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="G32" s="23" t="s">
+      <c r="E32" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="H32" s="21" t="s">
+      <c r="F32" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="I32" s="21" t="s">
-        <v>175</v>
+      <c r="G32" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="H32" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="I32" s="28" t="s">
+        <v>174</v>
       </c>
       <c r="J32" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K32" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L32" s="16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="69.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B33" s="55" t="s">
-        <v>211</v>
-      </c>
-      <c r="C33" s="25"/>
-      <c r="D33" s="26" t="s">
-        <v>176</v>
-      </c>
-      <c r="E33" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="F33" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="G33" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="I33" s="26" t="s">
-        <v>179</v>
+        <v>207</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="C33" s="19"/>
+      <c r="D33" s="26">
+        <v>4</v>
+      </c>
+      <c r="E33" s="26">
+        <v>8</v>
+      </c>
+      <c r="F33" s="31">
+        <v>12</v>
+      </c>
+      <c r="G33" s="32">
+        <v>24</v>
+      </c>
+      <c r="H33" s="26">
+        <v>36</v>
+      </c>
+      <c r="I33" s="26">
+        <v>4</v>
       </c>
       <c r="J33" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K33" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L33" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B34" s="54" t="s">
-        <v>212</v>
-      </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C34" s="33"/>
+      <c r="D34" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>179</v>
+      </c>
+      <c r="F34" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="G34" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="H34" s="34" t="s">
         <v>182</v>
       </c>
-      <c r="F34" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="I34" s="13" t="s">
-        <v>182</v>
+      <c r="I34" s="34" t="s">
+        <v>178</v>
       </c>
       <c r="J34" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K34" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L34" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="70.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="105" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B35" s="54" t="s">
-        <v>213</v>
-      </c>
-      <c r="C35" s="19"/>
-      <c r="D35" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>203</v>
+      </c>
+      <c r="C35" s="36"/>
+      <c r="D35" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="E35" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="G35" s="26" t="s">
         <v>186</v>
       </c>
-      <c r="E35" s="28" t="s">
+      <c r="H35" s="26" t="s">
         <v>187</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="G35" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="H35" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="28" t="s">
-        <v>187</v>
+      <c r="I35" s="26" t="s">
+        <v>183</v>
       </c>
       <c r="J35" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K35" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L35" s="16">
+        <v>123</v>
+      </c>
+      <c r="L35" s="37">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="69.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B36" s="54" t="s">
-        <v>214</v>
-      </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="26">
-        <v>4</v>
-      </c>
-      <c r="E36" s="26">
-        <v>8</v>
-      </c>
-      <c r="F36" s="31">
-        <v>12</v>
-      </c>
-      <c r="G36" s="32">
-        <v>24</v>
-      </c>
-      <c r="H36" s="26">
-        <v>36</v>
-      </c>
-      <c r="I36" s="26">
-        <v>4</v>
+        <v>207</v>
+      </c>
+      <c r="B36" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="C36" s="37"/>
+      <c r="D36" s="38">
+        <v>0.08</v>
+      </c>
+      <c r="E36" s="38">
+        <v>0.16</v>
+      </c>
+      <c r="F36" s="38">
+        <v>0.32</v>
+      </c>
+      <c r="G36" s="38">
+        <v>0.64</v>
+      </c>
+      <c r="H36" s="38">
+        <v>0.96</v>
+      </c>
+      <c r="I36" s="38">
+        <v>0.32</v>
       </c>
       <c r="J36" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K36" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L36" s="16">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B37" s="56" t="s">
+    <row r="37" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="34" t="s">
-        <v>191</v>
-      </c>
-      <c r="E37" s="35" t="s">
-        <v>192</v>
-      </c>
-      <c r="F37" s="34" t="s">
-        <v>193</v>
-      </c>
-      <c r="G37" s="35" t="s">
-        <v>194</v>
-      </c>
-      <c r="H37" s="34" t="s">
-        <v>195</v>
-      </c>
-      <c r="I37" s="34" t="s">
-        <v>191</v>
+      <c r="C37" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="F37" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="G37" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="H37" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="I37" s="23" t="s">
+        <v>153</v>
       </c>
       <c r="J37" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K37" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L37" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="G38" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B38" s="57" t="s">
-        <v>216</v>
-      </c>
-      <c r="C38" s="36"/>
-      <c r="D38" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="F38" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="G38" s="26" t="s">
-        <v>199</v>
-      </c>
-      <c r="H38" s="26" t="s">
-        <v>200</v>
-      </c>
-      <c r="I38" s="26" t="s">
-        <v>196</v>
+      <c r="H38" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>218</v>
       </c>
       <c r="J38" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K38" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L38" s="37">
+        <v>123</v>
+      </c>
+      <c r="L38" s="16">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="B39" s="52" t="s">
-        <v>217</v>
-      </c>
-      <c r="C39" s="37"/>
-      <c r="D39" s="38">
-        <v>0.08</v>
-      </c>
-      <c r="E39" s="38">
-        <v>0.16</v>
-      </c>
-      <c r="F39" s="38">
-        <v>0.32</v>
-      </c>
-      <c r="G39" s="38">
-        <v>0.64</v>
-      </c>
-      <c r="H39" s="38">
-        <v>0.96</v>
-      </c>
-      <c r="I39" s="38">
-        <v>0.32</v>
+    <row r="39" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="C39" s="3"/>
+      <c r="D39" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="E39" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="F39" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="G39" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="H39" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="I39" s="23" t="s">
+        <v>212</v>
       </c>
       <c r="J39" s="15" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="K39" s="15" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="L39" s="16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="59" t="s">
-        <v>220</v>
-      </c>
-      <c r="B40" t="s">
-        <v>229</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="F40" s="23" t="s">
-        <v>168</v>
-      </c>
-      <c r="G40" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="H40" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="I40" s="23" t="s">
-        <v>166</v>
+      <c r="A40" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B40" s="46" t="s">
+        <v>235</v>
+      </c>
+      <c r="C40" s="3"/>
+      <c r="D40" s="46" t="s">
+        <v>239</v>
+      </c>
+      <c r="E40" s="46" t="s">
+        <v>240</v>
+      </c>
+      <c r="F40" s="46" t="s">
+        <v>241</v>
+      </c>
+      <c r="G40" s="46" t="s">
+        <v>242</v>
+      </c>
+      <c r="H40" s="46" t="s">
+        <v>243</v>
+      </c>
+      <c r="I40" s="46" t="s">
+        <v>239</v>
       </c>
       <c r="J40" s="15" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="L40" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="59" t="s">
-        <v>220</v>
-      </c>
-      <c r="B41" t="s">
-        <v>223</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>224</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>226</v>
-      </c>
-      <c r="G41" s="23" t="s">
-        <v>227</v>
-      </c>
-      <c r="H41" s="21" t="s">
-        <v>228</v>
-      </c>
-      <c r="I41" s="23" t="s">
-        <v>226</v>
+      <c r="A41" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B41" s="46" t="s">
+        <v>236</v>
+      </c>
+      <c r="C41" s="3"/>
+      <c r="D41" s="46" t="s">
+        <v>256</v>
+      </c>
+      <c r="E41" s="46" t="s">
+        <v>255</v>
+      </c>
+      <c r="F41" s="46" t="s">
+        <v>257</v>
+      </c>
+      <c r="G41" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="H41" s="46" t="s">
+        <v>244</v>
+      </c>
+      <c r="I41" s="46" t="s">
+        <v>257</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="L41" s="16">
         <v>1</v>
       </c>
+    </row>
+    <row r="42" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B42" s="46" t="s">
+        <v>237</v>
+      </c>
+      <c r="C42" s="3"/>
+      <c r="D42" s="46" t="s">
+        <v>303</v>
+      </c>
+      <c r="E42" s="46" t="s">
+        <v>302</v>
+      </c>
+      <c r="F42" s="46" t="s">
+        <v>259</v>
+      </c>
+      <c r="G42" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="H42" s="46" t="s">
+        <v>304</v>
+      </c>
+      <c r="I42" s="46" t="s">
+        <v>304</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K42" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L42" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B43" s="46" t="s">
+        <v>238</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="46" t="s">
+        <v>261</v>
+      </c>
+      <c r="E43" s="46" t="s">
+        <v>262</v>
+      </c>
+      <c r="F43" s="46" t="s">
+        <v>245</v>
+      </c>
+      <c r="G43" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="H43" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="I43" s="46" t="s">
+        <v>263</v>
+      </c>
+      <c r="J43" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K43" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L43" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A44" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B44" s="46" t="s">
+        <v>223</v>
+      </c>
+      <c r="C44" s="3"/>
+      <c r="D44" s="46" t="s">
+        <v>224</v>
+      </c>
+      <c r="E44" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="F44" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="G44" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="H44" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="I44" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="J44" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K44" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L44" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A45" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B45" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="E45" s="46" t="s">
+        <v>265</v>
+      </c>
+      <c r="F45" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="G45" s="46" t="s">
+        <v>267</v>
+      </c>
+      <c r="H45" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="I45" s="46" t="s">
+        <v>230</v>
+      </c>
+      <c r="J45" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K45" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L45" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A46" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B46" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="C46" s="3"/>
+      <c r="D46" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="E46" s="46" t="s">
+        <v>268</v>
+      </c>
+      <c r="F46" s="46" t="s">
+        <v>269</v>
+      </c>
+      <c r="G46" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="H46" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="I46" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="J46" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K46" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L46" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A47" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B47" s="46" t="s">
+        <v>232</v>
+      </c>
+      <c r="C47" s="3"/>
+      <c r="D47" s="46" t="s">
+        <v>271</v>
+      </c>
+      <c r="E47" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="F47" s="46" t="s">
+        <v>273</v>
+      </c>
+      <c r="G47" s="46" t="s">
+        <v>301</v>
+      </c>
+      <c r="H47" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="I47" s="46" t="s">
+        <v>273</v>
+      </c>
+      <c r="J47" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K47" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L47" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A48" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B48" s="46" t="s">
+        <v>234</v>
+      </c>
+      <c r="C48" s="3"/>
+      <c r="D48" s="46" t="s">
+        <v>275</v>
+      </c>
+      <c r="E48" s="46" t="s">
+        <v>276</v>
+      </c>
+      <c r="F48" s="46" t="s">
+        <v>277</v>
+      </c>
+      <c r="G48" s="46" t="s">
+        <v>299</v>
+      </c>
+      <c r="H48" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="I48" s="46" t="s">
+        <v>277</v>
+      </c>
+      <c r="J48" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K48" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L48" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B49" s="46" t="s">
+        <v>247</v>
+      </c>
+      <c r="C49" s="3"/>
+      <c r="D49" s="46" t="s">
+        <v>279</v>
+      </c>
+      <c r="E49" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="F49" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="G49" s="46" t="s">
+        <v>278</v>
+      </c>
+      <c r="H49" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="I49" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="J49" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K49" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L49" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B50" s="46" t="s">
+        <v>248</v>
+      </c>
+      <c r="C50" s="3"/>
+      <c r="D50" s="46" t="s">
+        <v>250</v>
+      </c>
+      <c r="E50" s="46" t="s">
+        <v>251</v>
+      </c>
+      <c r="F50" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="G50" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="H50" s="46" t="s">
+        <v>284</v>
+      </c>
+      <c r="I50" s="46" t="s">
+        <v>282</v>
+      </c>
+      <c r="J50" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K50" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L50" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A51" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B51" s="46" t="s">
+        <v>285</v>
+      </c>
+      <c r="C51" s="3"/>
+      <c r="D51" s="46" t="s">
+        <v>286</v>
+      </c>
+      <c r="E51" s="46" t="s">
+        <v>294</v>
+      </c>
+      <c r="F51" s="46" t="s">
+        <v>295</v>
+      </c>
+      <c r="G51" s="46" t="s">
+        <v>296</v>
+      </c>
+      <c r="H51" s="46" t="s">
+        <v>297</v>
+      </c>
+      <c r="I51" s="46" t="s">
+        <v>286</v>
+      </c>
+      <c r="J51" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K51" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L51" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="150" x14ac:dyDescent="0.25">
+      <c r="A52" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B52" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="C52" s="3"/>
+      <c r="D52" s="46" t="s">
+        <v>293</v>
+      </c>
+      <c r="E52" s="46" t="s">
+        <v>305</v>
+      </c>
+      <c r="F52" s="46" t="s">
+        <v>292</v>
+      </c>
+      <c r="G52" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="H52" s="46" t="s">
+        <v>253</v>
+      </c>
+      <c r="I52" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="J52" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K52" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L52" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A53" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B53" s="46" t="s">
+        <v>291</v>
+      </c>
+      <c r="C53" s="3"/>
+      <c r="D53" s="46" t="s">
+        <v>287</v>
+      </c>
+      <c r="E53" s="46" t="s">
+        <v>288</v>
+      </c>
+      <c r="F53" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="G53" s="46" t="s">
+        <v>290</v>
+      </c>
+      <c r="H53" s="46" t="s">
+        <v>254</v>
+      </c>
+      <c r="I53" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="J53" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K53" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="L53" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B54" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="C54" s="3"/>
+      <c r="D54" s="46" t="s">
+        <v>320</v>
+      </c>
+      <c r="E54" s="46" t="s">
+        <v>321</v>
+      </c>
+      <c r="F54" s="46" t="s">
+        <v>322</v>
+      </c>
+      <c r="G54" s="46" t="s">
+        <v>323</v>
+      </c>
+      <c r="H54" s="46" t="s">
+        <v>324</v>
+      </c>
+      <c r="I54" s="46" t="s">
+        <v>322</v>
+      </c>
+      <c r="J54" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K54" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L54" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B55" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="C55" s="3"/>
+      <c r="D55" s="46" t="s">
+        <v>325</v>
+      </c>
+      <c r="E55" s="46" t="s">
+        <v>326</v>
+      </c>
+      <c r="F55" s="46" t="s">
+        <v>327</v>
+      </c>
+      <c r="G55" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="H55" s="46" t="s">
+        <v>329</v>
+      </c>
+      <c r="I55" s="46" t="s">
+        <v>325</v>
+      </c>
+      <c r="J55" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K55" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L55" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B56" s="46" t="s">
+        <v>309</v>
+      </c>
+      <c r="C56" s="3"/>
+      <c r="D56" s="46" t="s">
+        <v>330</v>
+      </c>
+      <c r="E56" s="46" t="s">
+        <v>331</v>
+      </c>
+      <c r="F56" s="46" t="s">
+        <v>332</v>
+      </c>
+      <c r="G56" s="46" t="s">
+        <v>333</v>
+      </c>
+      <c r="H56" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I56" s="46" t="s">
+        <v>333</v>
+      </c>
+      <c r="J56" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K56" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L56" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A57" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B57" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="C57" s="3"/>
+      <c r="D57" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="E57" s="46" t="s">
+        <v>336</v>
+      </c>
+      <c r="F57" s="46" t="s">
+        <v>337</v>
+      </c>
+      <c r="G57" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="H57" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I57" s="46" t="s">
+        <v>336</v>
+      </c>
+      <c r="J57" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K57" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L57" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A58" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B58" s="46" t="s">
+        <v>311</v>
+      </c>
+      <c r="C58" s="3"/>
+      <c r="D58" s="46" t="s">
+        <v>339</v>
+      </c>
+      <c r="E58" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="F58" s="46" t="s">
+        <v>341</v>
+      </c>
+      <c r="G58" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="H58" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I58" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="J58" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K58" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L58" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A59" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B59" s="46" t="s">
+        <v>374</v>
+      </c>
+      <c r="C59" s="3"/>
+      <c r="D59" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="E59" s="46" t="s">
+        <v>343</v>
+      </c>
+      <c r="F59" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="G59" s="46" t="s">
+        <v>345</v>
+      </c>
+      <c r="H59" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I59" s="46" t="s">
+        <v>343</v>
+      </c>
+      <c r="J59" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K59" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L59" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A60" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B60" s="46" t="s">
+        <v>312</v>
+      </c>
+      <c r="C60" s="3"/>
+      <c r="D60" s="46" t="s">
+        <v>339</v>
+      </c>
+      <c r="E60" s="46" t="s">
+        <v>346</v>
+      </c>
+      <c r="F60" s="46" t="s">
+        <v>347</v>
+      </c>
+      <c r="G60" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="H60" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I60" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="J60" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K60" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L60" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B61" s="46" t="s">
+        <v>313</v>
+      </c>
+      <c r="C61" s="3"/>
+      <c r="D61" s="46" t="s">
+        <v>348</v>
+      </c>
+      <c r="E61" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="F61" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="G61" s="46" t="s">
+        <v>351</v>
+      </c>
+      <c r="H61" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I61" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="J61" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K61" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L61" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="120" x14ac:dyDescent="0.25">
+      <c r="A62" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B62" s="46" t="s">
+        <v>314</v>
+      </c>
+      <c r="C62" s="3"/>
+      <c r="D62" s="46" t="s">
+        <v>352</v>
+      </c>
+      <c r="E62" s="46" t="s">
+        <v>353</v>
+      </c>
+      <c r="F62" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="G62" s="46" t="s">
+        <v>355</v>
+      </c>
+      <c r="H62" s="46" t="s">
+        <v>356</v>
+      </c>
+      <c r="I62" s="46" t="s">
+        <v>355</v>
+      </c>
+      <c r="J62" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K62" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L62" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B63" s="46" t="s">
+        <v>315</v>
+      </c>
+      <c r="C63" s="3"/>
+      <c r="D63" s="46" t="s">
+        <v>357</v>
+      </c>
+      <c r="E63" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="F63" s="46" t="s">
+        <v>359</v>
+      </c>
+      <c r="G63" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="H63" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I63" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="J63" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K63" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L63" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A64" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B64" s="46" t="s">
+        <v>316</v>
+      </c>
+      <c r="C64" s="3"/>
+      <c r="D64" s="46" t="s">
+        <v>361</v>
+      </c>
+      <c r="E64" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="F64" s="46" t="s">
+        <v>363</v>
+      </c>
+      <c r="G64" s="46" t="s">
+        <v>364</v>
+      </c>
+      <c r="H64" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I64" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="J64" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K64" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L64" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A65" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B65" s="46" t="s">
+        <v>317</v>
+      </c>
+      <c r="C65" s="3"/>
+      <c r="D65" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="E65" s="46" t="s">
+        <v>365</v>
+      </c>
+      <c r="F65" s="46" t="s">
+        <v>341</v>
+      </c>
+      <c r="G65" s="46" t="s">
+        <v>366</v>
+      </c>
+      <c r="H65" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I65" s="46" t="s">
+        <v>335</v>
+      </c>
+      <c r="J65" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K65" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L65" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B66" s="46" t="s">
+        <v>318</v>
+      </c>
+      <c r="C66" s="3"/>
+      <c r="D66" s="46" t="s">
+        <v>367</v>
+      </c>
+      <c r="E66" s="46" t="s">
+        <v>368</v>
+      </c>
+      <c r="F66" s="46" t="s">
+        <v>369</v>
+      </c>
+      <c r="G66" s="46" t="s">
+        <v>370</v>
+      </c>
+      <c r="H66" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I66" s="46" t="s">
+        <v>368</v>
+      </c>
+      <c r="J66" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K66" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L66" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B67" s="46" t="s">
+        <v>319</v>
+      </c>
+      <c r="C67" s="3"/>
+      <c r="D67" s="46" t="s">
+        <v>371</v>
+      </c>
+      <c r="E67" s="46" t="s">
+        <v>372</v>
+      </c>
+      <c r="F67" s="46" t="s">
+        <v>373</v>
+      </c>
+      <c r="G67" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="H67" s="46" t="s">
+        <v>334</v>
+      </c>
+      <c r="I67" s="46" t="s">
+        <v>373</v>
+      </c>
+      <c r="J67" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="K67" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="L67" s="47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B68" s="48" t="s">
+        <v>375</v>
+      </c>
+      <c r="C68" s="48" t="s">
+        <v>376</v>
+      </c>
+      <c r="J68" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="K68" s="42" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B69" s="48" t="s">
+        <v>377</v>
+      </c>
+      <c r="D69" s="48" t="s">
+        <v>378</v>
+      </c>
+      <c r="E69" s="48" t="s">
+        <v>379</v>
+      </c>
+      <c r="F69" s="49" t="s">
+        <v>380</v>
+      </c>
+      <c r="G69" s="49" t="s">
+        <v>381</v>
+      </c>
+      <c r="H69" s="49" t="s">
+        <v>382</v>
+      </c>
+      <c r="L69" s="50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B70" s="48"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>